<commit_message>
단위검증 TC 추가- UpdateOutpus()
</commit_message>
<xml_diff>
--- a/projects/embeded-power-manager/test/UnitTest_TC.xlsx
+++ b/projects/embeded-power-manager/test/UnitTest_TC.xlsx
@@ -19,13 +19,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
-  <x:si>
-    <x:t>Init() 수행시 시스템이 초기 상태로 초기화되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1. PowerManager 객체 생성
-2. Init() 호출</x:t>
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="76">
+  <x:si>
+    <x:t>Current State = ACTIVE
+IGN Signal = FALSE</x:t>
   </x:si>
   <x:si>
     <x:t>Current State가 POWER_OFF로 설정된다.
@@ -36,6 +33,29 @@
 Timer가 초기화된다.</x:t>
   </x:si>
   <x:si>
+    <x:t>UT-EPM-012</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. Current State를 LOW_POWER로 설정
+2. UpdateOutputs()를 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = INIT
+Initialization Complete = TRUE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = FAULT
+CAN Message = RESET_FAULT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = SLEEP
+IGN Signal = TRUE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = SLEEP
+Sleep Timer = 30s</x:t>
+  </x:si>
+  <x:si>
     <x:t>LOW_POWER 상태에서 배터리 전압이 정상 전압으로 복구되면 ACTIVE 상태로 전이되는지 확인한다.</x:t>
   </x:si>
   <x:si>
@@ -43,86 +63,123 @@
 isInitFinished가 false로 변경된다. </x:t>
   </x:si>
   <x:si>
+    <x:t>1. PowerManager 객체 생성
+2. Init() 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Init() 수행시 시스템이 초기 상태로 초기화되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = ACTIVE
+Battery Voltage = 9.9V</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LOW_POWER 상태에서 주변 장치 및 카메라 전원이 올바르게 설정되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. Current State를 POWER_OFF로 설정
+2. UpdateOutputs()를 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. RecvCanMessage(RESET_FAULT) 호출
+2. UpdateState() 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACTIVE 상태에서 Battery Fault 발생 시 FAULT 상태로 전이되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. SetBatteryVoltage(9.9) 호출
+2. UpdateState() 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. SetBatteryVoltage(11.5) 호출
+2. UpdateState() 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FAULT 상태에서 Fault Reset 명령 수신 시 INIT 상태로 전이되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACTIVE 상태에서 배터리 전압이 낮아지면 LOW_POWER 상태로 전이되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. SetBatteryVoltage(11.4) 호출
+2. UpdateState() 호출</x:t>
+  </x:si>
+  <x:si>
     <x:t>1. SetIgnSignal(true) 호출
 2. UpdateState() 호출</x:t>
   </x:si>
   <x:si>
+    <x:t>SLEEP 상태에서 Wakeup 요청이 오면 INIT 상태로 전이되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
     <x:t>SLEEP 상태에서 30초 경과되면 POWE_OFF 상태로 전이되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INIT 상태에서 초기화 완료 시 시스템 상태가 ACTIVE로 전이되는지 확인한다.</x:t>
   </x:si>
   <x:si>
     <x:t>1. SetInitFinished(true) 호출
 2. UpdateState() 호출</x:t>
   </x:si>
   <x:si>
-    <x:t>SLEEP 상태에서 Wakeup 요청이 오면 INIT 상태로 전이되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACTIVE 상태에서 IGN OFF 입력 시 SLEEP 상태로 전이되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
     <x:t>1. SetIgnSignal(false) 호출
 2. UpdateState() 호출</x:t>
   </x:si>
   <x:si>
-    <x:t>1. SetBatteryVoltage(9.9) 호출
-2. UpdateState() 호출</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FAULT 상태에서 Fault Reset 명령 수신 시 INIT 상태로 전이되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1. SetBatteryVoltage(11.5) 호출
-2. UpdateState() 호출</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACTIVE 상태에서 배터리 전압이 낮아지면 LOW_POWER 상태로 전이되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1. SetBatteryVoltage(11.4) 호출
-2. UpdateState() 호출</x:t>
+    <x:t>INIT 상태에서 초기화 완료 시 시스템 상태가 ACTIVE로 전이되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACTIVE 상태에서 IGN OFF 입력 시 SLEEP 상태로 전이되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>N/A</x:t>
   </x:si>
   <x:si>
     <x:t>IGN ON 입력 시 시스템 상태가 POWER_OFF에서 INIT으로 전이되는지 확인한다.</x:t>
   </x:si>
   <x:si>
+    <x:t>Current State = LOW_POWER
+Battery Voltage = 11.5V</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UpdateOutputs()</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UT-EPM-002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UT-EPM-001</x:t>
+  </x:si>
+  <x:si>
     <x:t>UT-EPM-007</x:t>
   </x:si>
   <x:si>
-    <x:t>UT-EPM-001</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UT-EPM-002</x:t>
-  </x:si>
-  <x:si>
     <x:t>UT-EPM-003</x:t>
   </x:si>
   <x:si>
+    <x:t>UT-EPM-009</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UT-EPM-004</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UT-EPM-006</x:t>
+  </x:si>
+  <x:si>
     <x:t>UT-EPM-008</x:t>
   </x:si>
   <x:si>
-    <x:t>UT-EPM-006</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UT-EPM-004</x:t>
+    <x:t>UT-EPM-010</x:t>
   </x:si>
   <x:si>
     <x:t>UT-EPM-005</x:t>
   </x:si>
   <x:si>
-    <x:t>UT-EPM-009</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UT-EPM-010</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACTIVE 상태에서 Battery Fault 발생 시 FAULT 상태로 전이되는지 확인한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1. RecvCanMessage(RESET_FAULT) 호출
-2. UpdateState() 호출</x:t>
+    <x:t>UT-EPM-011</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SDD-EPM-003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State가 SLEEP으로 변경된다.</x:t>
   </x:si>
   <x:si>
     <x:t>Current State가 ACTIVE로 변경된다.</x:t>
@@ -131,64 +188,21 @@
     <x:t>Current State가 LOW_POWER로 변경된다.</x:t>
   </x:si>
   <x:si>
-    <x:t>Initialization Complete = TRUE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State가 SLEEP으로 변경된다.</x:t>
-  </x:si>
-  <x:si>
     <x:t>Current State가 POWER_OFF로 변경된다.</x:t>
   </x:si>
   <x:si>
-    <x:t>IGN Signal = FALSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sleep Timer = 30s</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IGN Signal = TRUE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>N/A</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Battery Voltage = 11.5V</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Battery Voltage = 9.9V</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State = SLEEP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State = ACTIVE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State = INIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State = FAULT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Battery Voltage = 11.4V</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State가 FAULT로 변경된다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CAN Message = RESET_FAULT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State = POWER_OFF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State가 INIT으로 변경된다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>추후 sleepTimert설정하는 설계 필요</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Current State = LOW_POWER</x:t>
+    <x:t>Peripheral Power Enable = FALSE
+Camera Power Enable = FALSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">SDD-EPM-002
+</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UpdateState()</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Test Purpose</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SDD-EPM-001
@@ -198,41 +212,72 @@
     <x:t>Test Function</x:t>
   </x:si>
   <x:si>
-    <x:t>UpdateState()</x:t>
+    <x:t>Test Procedure</x:t>
   </x:si>
   <x:si>
     <x:t>Pre-condition</x:t>
   </x:si>
   <x:si>
-    <x:t>Test Procedure</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Test Purpose</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SDD-EPM-002
-</x:t>
+    <x:t>SDD ID</x:t>
   </x:si>
   <x:si>
     <x:t>Output</x:t>
   </x:si>
   <x:si>
+    <x:t>Init()</x:t>
+  </x:si>
+  <x:si>
     <x:t>TC ID</x:t>
   </x:si>
   <x:si>
-    <x:t>Init()</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SDD ID</x:t>
-  </x:si>
-  <x:si>
     <x:t>Input</x:t>
   </x:si>
   <x:si>
-    <x:t>UT-EPM-011</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SDD-EPM-003</x:t>
+    <x:t>추후 sleepTimert설정하는 설계 필요</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = POWER_OFF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State가 INIT으로 변경된다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State가 FAULT로 변경된다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = ACTIVE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UT-EPM-013</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = ACTIVE
+Battery Voltage = 11.4V</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = LOW_POWER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Current State = POWER_OFF
+IGN Signal = TRUE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>POWER_OFF 상태에서주변 장치 및 카메라 전원이 올바르게 설정되는지 확인한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1. Current State를 ACTIVE로 설정
+2. UpdateOutputs()를 호출</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Peripheral Power Enable = TRUE
+Camera Power Enable = FALSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Peripheral Power Enable = TRUE
+Camera Power Enable = TRUE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACTIVE 상태에서주변 장치 및 카메라 전원이 올바르게 설정되는지 확인한다.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -705,15 +750,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:K12"/>
+  <x:dimension ref="A1:K15"/>
   <x:sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.399999999999999"/>
   <x:cols>
     <x:col min="1" max="1" width="11.89453125" style="2" bestFit="1" customWidth="1"/>
     <x:col min="2" max="2" width="13.41015625" style="2" bestFit="1" customWidth="1"/>
     <x:col min="3" max="3" width="83.73046875" style="1" bestFit="1" customWidth="1"/>
     <x:col min="4" max="4" width="12.74609375" style="2" bestFit="1" customWidth="1"/>
-    <x:col min="5" max="5" width="26.3671875" style="2" bestFit="1" customWidth="1"/>
-    <x:col min="6" max="6" width="26.56640625" style="2" bestFit="1" customWidth="1"/>
+    <x:col min="5" max="5" width="12.12109375" style="2" bestFit="1" customWidth="1"/>
+    <x:col min="6" max="6" width="27.25" style="2" customWidth="1"/>
     <x:col min="7" max="7" width="34.87890625" style="2" bestFit="1" customWidth="1"/>
     <x:col min="8" max="8" width="36.9609375" style="2" bestFit="1" customWidth="1"/>
   </x:cols>
@@ -723,300 +768,375 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B1" s="5" t="s">
-        <x:v>62</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C1" s="5" t="s">
-        <x:v>57</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D1" s="5" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E1" s="5" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="G1" s="5" t="s">
-        <x:v>56</x:v>
-      </x:c>
       <x:c r="H1" s="5" t="s">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8" ht="98.25">
       <x:c r="A2" s="4" t="s">
-        <x:v>19</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B2" s="7" t="s">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C2" s="7" t="s">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D2" s="4" t="s">
-        <x:v>61</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F2" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="G2" s="6" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="s">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="H2" s="6" t="s">
-        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8" ht="32.75">
       <x:c r="A3" s="4" t="s">
-        <x:v>20</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B3" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C3" s="8" t="s">
-        <x:v>17</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D3" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E3" s="4" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="F3" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="s">
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G3" s="6" t="s">
-        <x:v>5</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H3" s="4" t="s">
-        <x:v>49</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8" ht="32.75">
       <x:c r="A4" s="4" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B4" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C4" s="8" t="s">
-        <x:v>7</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E4" s="4" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F4" s="8" t="s">
-        <x:v>32</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="s">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G4" s="6" t="s">
-        <x:v>8</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H4" s="6" t="s">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:8" ht="32.75">
       <x:c r="A5" s="4" t="s">
-        <x:v>24</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B5" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C5" s="4" t="s">
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>45</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="s">
+        <x:v>68</x:v>
       </x:c>
       <x:c r="G5" s="6" t="s">
-        <x:v>16</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H5" s="6" t="s">
-        <x:v>31</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:11" ht="32.75">
       <x:c r="A6" s="4" t="s">
-        <x:v>25</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s">
-        <x:v>10</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E6" s="4" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F6" s="4" t="s">
-        <x:v>35</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="s">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="6" t="s">
-        <x:v>11</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="H6" s="6" t="s">
-        <x:v>33</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:8" ht="32.75">
       <x:c r="A7" s="4" t="s">
-        <x:v>23</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C7" s="4" t="s">
-        <x:v>3</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E7" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:8" ht="32.75">
+      <x:c r="A8" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="G7" s="6" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="H7" s="6" t="s">
-        <x:v>30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:8">
-      <x:c r="A8" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="C8" s="4" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D8" s="4" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="E8" s="4" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F8" s="4" t="s">
-        <x:v>36</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="s">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G8" s="4" t="s">
-        <x:v>50</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="H8" s="6" t="s">
-        <x:v>34</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:8" ht="32.75">
       <x:c r="A9" s="4" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="C9" s="4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="D9" s="4" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F9" s="4" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G9" s="6" t="s">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="H9" s="6" t="s">
-        <x:v>49</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:8" ht="32.75">
       <x:c r="A10" s="4" t="s">
-        <x:v>26</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B10" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C10" s="6" t="s">
-        <x:v>28</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D10" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E10" s="4" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F10" s="4" t="s">
-        <x:v>40</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="s">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G10" s="6" t="s">
-        <x:v>12</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H10" s="6" t="s">
-        <x:v>46</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:8" ht="32.75">
       <x:c r="A11" s="4" t="s">
-        <x:v>27</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C11" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="s">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:8" ht="32.75">
+      <x:c r="A12" s="4" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:8" customFormat="1" ht="32.75">
+      <x:c r="A13" s="4" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:8" ht="32.75">
+      <x:c r="A14" s="4" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F11" s="4" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="G11" s="6" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="H11" s="6" t="s">
-        <x:v>49</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:8">
-      <x:c r="A12" s="1" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="B12" s="1" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="D12" s="1"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
-      <x:c r="G12" s="1"/>
-      <x:c r="H12" s="1"/>
+      <x:c r="D14" s="4" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="s">
+        <x:v>73</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:8">
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>

</xml_diff>